<commit_message>
Import Excel answers as confirmed primary information
</commit_message>
<xml_diff>
--- a/public/primary-information-template.xlsx
+++ b/public/primary-information-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一次情報入力" sheetId="1" r:id="R6c1ee3b158424bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一次情報入力" sheetId="1" r:id="Rec4aa956102644fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -92,42 +92,12 @@
   </x:fills>
   <x:borders count="7">
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -362,7 +332,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>B列に、分かる範囲でそのまま入力してください。文章でも箇条書きでも大丈夫です。入力後はPDFにして、SEO LOOPの「一次情報」に追加します。</x:v>
+        <x:v>B列に、分かる範囲で入力してください。文章でも箇条書きでも大丈夫です。入力後はExcel形式（.xlsx）のまま、SEO LOOPの「一次情報」へ追加します。</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
     </x:row>
@@ -436,7 +406,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="18" t="str">
-        <x:v>PDFにする方法：入力後に、Excelの「ファイル」→「エクスポート」または「名前を付けて保存」からPDFを選びます。できたPDFをSEO LOOPの一次情報ページへ追加してください。</x:v>
+        <x:v>追加方法：B列に回答を入力してExcel形式（.xlsx）で保存し、SEO LOOPの一次情報ページからファイルを追加してください。読み取った原文を確認してから記事利用を確定します。</x:v>
       </x:c>
       <x:c r="B16" s="18"/>
     </x:row>

</xml_diff>